<commit_message>
audit log slot 5
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenThiThuyTien.xlsx
+++ b/AI Audit Log_NguyenThiThuyTien.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nguyenthithuytien/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nguyenthithuytien/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44FD8D86-5B7C-9D40-BFFA-4AB9A8825EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755D849E-2EDF-1A40-B8AF-D0072DC3A186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="28480" windowHeight="15820" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="28480" windowHeight="15820" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
-    <sheet name="Assignment 1" sheetId="2" r:id="rId2"/>
+    <sheet name="Week 2" sheetId="1" r:id="rId1"/>
+    <sheet name="Week 3" sheetId="2" r:id="rId2"/>
     <sheet name="Assignment 2" sheetId="3" r:id="rId3"/>
     <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
   </sheets>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="44">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -381,6 +381,434 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> Tôi đổi lại một số tên use case để thống nhất cách đặt tên và dễ hiểu hơn khi trình bày.</t>
+    </r>
+  </si>
+  <si>
+    <t>Slot 5</t>
+  </si>
+  <si>
+    <t>“Trong hệ thống quản lý thư viện online, nên xác định các Entity chính như thế nào để tránh thiếu class khi vẽ UML?”</t>
+  </si>
+  <si>
+    <t>“Ở giai đoạn phân tích hệ thống, có cần thêm DAO hoặc Repository vào Class Diagram không?”</t>
+  </si>
+  <si>
+    <t>“Nên biểu diễn Interface trong UML như thế nào để đúng chuẩn?”</t>
+  </si>
+  <si>
+    <t>“Sequence Diagram có cần hiển thị đầy đủ Database hay không?”</t>
+  </si>
+  <si>
+    <t>“Khi nào nên dùng Activity Diagram thay vì Sequence Diagram?”</t>
+  </si>
+  <si>
+    <t>“Trong Use Case Diagram, chức năng Login nên include hay extend với Register?”</t>
+  </si>
+  <si>
+    <t>“Có nên đưa Validation vào Sequence Diagram không?”</t>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI đề xuất các Entity cốt lõi gồm: Book, Author, Member, BorrowTicket, Librarian và Category. Đồng thời giải thích rằng Entity nên đại diện cho dữ liệu tồn tại lâu dài trong hệ thống.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Người học bổ sung thêm Reservation vì hệ thống có chức năng giữ sách trước.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>“Trong UML, multiplicity 0..</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 1..</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, và 1 khác nhau như thế nào?”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI giải thích: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> nghĩa là bắt buộc đúng một đối tượng; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>0..*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> là có thể không có hoặc có nhiều; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>1..*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> là phải có ít nhất một. AI cũng đưa ví dụ thực tế giữa Customer và Order.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Người học điều chỉnh multiplicity của Customer – Order từ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> thành </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>0..*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> để phù hợp nghiệp vụ khách chưa mua hàng vẫn có tài khoản.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI cho rằng nếu sơ đồ phục vụ phân tích nghiệp vụ thì chỉ nên tập trung vào Entity và quan hệ nghiệp vụ. DAO/Repository phù hợp hơn ở giai đoạn thiết kế chi tiết.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Người học giữ sơ đồ đơn giản ở mức domain model và để Repository sang sơ đồ thiết kế sau.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI hướng dẫn rằng Interface có thể dùng ký hiệu </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>&lt;&lt;interface&gt;&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> hoặc hình tròn lollipop. Quan hệ triển khai dùng nét đứt với mũi tên tam giác rỗng.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Người học áp dụng Interface cho PaymentService và EmailService để tăng tính mở rộng cho hệ thống.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI giải thích rằng Sequence Diagram chủ yếu mô tả luồng tương tác giữa actor và object. Database chỉ nên thêm nếu cần làm rõ quá trình truy vấn dữ liệu.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Người học chỉ giữ Repository thay vì vẽ trực tiếp Database để sơ đồ gọn hơn.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI phân tích rằng Activity Diagram phù hợp mô tả luồng nghiệp vụ tổng quát, còn Sequence Diagram tập trung vào thứ tự gọi hàm giữa các object.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Dùng Activity Diagram cho quy trình đặt vé và Sequence Diagram cho chức năng thanh toán.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI cho biết Login và Register là hai use case độc lập nên không cần include hoặc extend. Chỉ nên liên kết trực tiếp với Actor.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Người học tách riêng hai use case để tránh hiểu sai quan hệ chức năng.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Phản hồi:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI đề xuất chỉ nên thể hiện các bước validation quan trọng ảnh hưởng đến luồng xử lý chính, ví dụ kiểm tra dữ liệu rỗng hoặc xác thực tài khoản.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Quyết định:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="163"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Người học thêm bước validate login trước khi gọi AuthService để luồng xử lý thực tế hơn.</t>
     </r>
   </si>
 </sst>
@@ -388,7 +816,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -423,6 +851,30 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="163"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -461,7 +913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -486,6 +938,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -951,9 +1415,233 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E3EFE9-6FFB-49CC-BE69-0C0E36C6253E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" style="10"/>
+    <col min="2" max="2" width="31.33203125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="42.6640625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="52.6640625" style="9" customWidth="1"/>
+    <col min="5" max="16384" width="8.83203125" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="12">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="12">
+        <v>2</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="12">
+        <v>4</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="12">
+        <v>5</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="47" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="12">
+        <v>6</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A14" s="12">
+        <v>7</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+      <c r="A16" s="12">
+        <v>8</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>